<commit_message>
Update Privacy News Dashboard snapshot (2026-09-18 11:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/moleg_news.xlsx
+++ b/docs/snapshot/downloads/moleg_news.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,27 +461,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>31651</t>
+          <t>31861</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
+          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>경제법제국</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -491,39 +491,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -533,29 +533,29 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -565,7 +565,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -575,39 +575,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -617,39 +617,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -659,39 +659,39 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -701,39 +701,39 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -743,29 +743,29 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -797,27 +797,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -827,34 +827,34 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -869,39 +869,39 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -911,39 +911,39 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -953,39 +953,39 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -995,29 +995,29 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1049,27 +1049,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1079,34 +1079,34 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1121,39 +1121,39 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1163,39 +1163,39 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1205,39 +1205,39 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1247,39 +1247,39 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1289,39 +1289,39 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1331,29 +1331,29 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1385,27 +1385,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1427,27 +1427,27 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1469,27 +1469,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1511,27 +1511,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1553,27 +1553,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1595,27 +1595,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1637,27 +1637,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1679,40 +1679,82 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-10-01 10:20:02 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/moleg_news.xlsx
+++ b/docs/snapshot/downloads/moleg_news.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>36341</t>
+          <t>37152</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
+          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -481,7 +481,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -491,39 +491,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>33671</t>
+          <t>37151</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
+          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>법제조정법제관실</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -533,39 +533,39 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>33082</t>
+          <t>36341</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
+          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -575,39 +575,39 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>31861</t>
+          <t>33671</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
+          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>법제조정법제관실</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -617,39 +617,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>31651</t>
+          <t>33082</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
+          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>경제법제국</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -659,39 +659,39 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31861</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -701,39 +701,39 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -743,39 +743,39 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -785,39 +785,39 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -827,39 +827,39 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -869,39 +869,39 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -911,39 +911,39 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -953,39 +953,39 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -995,39 +995,39 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1037,39 +1037,39 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1079,39 +1079,39 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1121,39 +1121,39 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1163,39 +1163,39 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1205,39 +1205,39 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1247,39 +1247,39 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1289,39 +1289,39 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1331,39 +1331,39 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1373,39 +1373,39 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1415,39 +1415,39 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1457,39 +1457,39 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1499,39 +1499,39 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1541,39 +1541,39 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1595,27 +1595,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1637,27 +1637,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1679,27 +1679,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1721,27 +1721,27 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1763,27 +1763,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1805,27 +1805,27 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1847,40 +1847,124 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>혁신행정감사담당관실</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-10-02 11:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/moleg_news.xlsx
+++ b/docs/snapshot/downloads/moleg_news.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,17 +461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>37351</t>
+          <t>37581</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
+          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -481,7 +481,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -491,34 +491,34 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>37152</t>
+          <t>37351</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
+          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -533,29 +533,29 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>37151</t>
+          <t>37152</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
+          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -587,17 +587,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>36341</t>
+          <t>37151</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
+          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -617,39 +617,39 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>33671</t>
+          <t>36341</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
+          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>법제조정법제관실</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -659,39 +659,39 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>33082</t>
+          <t>33671</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
+          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>법제조정법제관실</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -701,29 +701,29 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>31861</t>
+          <t>33082</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
+          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -743,39 +743,39 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>31651</t>
+          <t>31861</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
+          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>경제법제국</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -785,39 +785,39 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -827,29 +827,29 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -869,39 +869,39 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -911,39 +911,39 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -953,39 +953,39 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -995,39 +995,39 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1037,29 +1037,29 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1091,27 +1091,27 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1121,34 +1121,34 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1163,39 +1163,39 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1205,39 +1205,39 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1247,39 +1247,39 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1289,29 +1289,29 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1343,27 +1343,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1373,34 +1373,34 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1415,39 +1415,39 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1457,39 +1457,39 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1499,39 +1499,39 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1541,39 +1541,39 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1583,39 +1583,39 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1625,29 +1625,29 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1679,27 +1679,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1721,27 +1721,27 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1763,27 +1763,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1805,27 +1805,27 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1847,27 +1847,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1889,27 +1889,27 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1931,27 +1931,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1973,40 +1973,82 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>

<commit_message>
Update Privacy News Dashboard snapshot (2026-10-02 14:20:01 KST)
</commit_message>
<xml_diff>
--- a/docs/snapshot/downloads/moleg_news.xlsx
+++ b/docs/snapshot/downloads/moleg_news.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,22 +461,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>37581</t>
+          <t>37711</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
+          <t>“행정기본법 제정 5주년, 새로운 길을 찾다”</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157976&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -491,29 +491,29 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-10-02 10:45:20.519914+09:00</t>
+          <t>2026-10-02 14:00:20.071730+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>37351</t>
+          <t>37581</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
+          <t>국민이 직접 뽑은 ‘대표 알기 쉬운 법령 용어’에 “사위(詐僞) → 거짓/속임수” 등 5개 선정</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157972&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -523,7 +523,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -533,34 +533,34 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-10-01 15:15:21.104965+09:00</t>
+          <t>2026-10-02 10:45:20.519914+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>37152</t>
+          <t>37351</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
+          <t>법제처, 알기 쉬운 법령 만들기 20년을 돌아보고 미래를 이야기하다!</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157915&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -575,29 +575,29 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-10-01 10:15:19.890918+09:00</t>
+          <t>2026-10-01 15:15:21.104965+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>37151</t>
+          <t>37152</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
+          <t>가상자산 활용 보이스피싱 피해 구제 확대 및 배달앱 원산지 표시 고지 의무화</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157902&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -629,17 +629,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>36341</t>
+          <t>37151</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
+          <t>Expanding Voice Phishing Damage Relief Utilizing Virtual Assets and ..</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157904&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -659,39 +659,39 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-29 10:30:21.085354+09:00</t>
+          <t>2026-10-01 10:15:19.890918+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>33671</t>
+          <t>36341</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
+          <t>법제처, AI로 국민과 법의 거리를 좁힌다</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157747&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>법제조정법제관실</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -701,39 +701,39 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-22 15:30:19.394844+09:00</t>
+          <t>2026-09-29 10:30:21.085354+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>33082</t>
+          <t>33671</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
+          <t>법제처, 인신매매 피해자의 권익 보호 강화를 위해 현장의 목소리를 듣다</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157435&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>법제조정법제관실</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -743,29 +743,29 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-21 11:00:21.026847+09:00</t>
+          <t>2026-09-22 15:30:19.394844+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>31861</t>
+          <t>33082</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
+          <t>MOLEG approves Nepal's accession to Council of Asian Legislative Institutions and ...</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -785,39 +785,39 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-18 11:15:19.901041+09:00</t>
+          <t>2026-09-21 11:00:21.026847+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>31651</t>
+          <t>31861</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
+          <t>법제처, 아시아 법제기구 협의체에 네팔 가입 승인 및 법 접근성 강화 관련 논의</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157225&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>경제법제국</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -827,39 +827,39 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-17 16:15:20.031512+09:00</t>
+          <t>2026-09-18 11:15:19.901041+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>31201</t>
+          <t>31651</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
+          <t>법제처, 전세사기피해자 주거안정 입법 조치를 위한 ‘찾아가는 법제심사’ 실시</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157176&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>경제법제국</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -869,29 +869,29 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-16 15:15:18.945495+09:00</t>
+          <t>2026-09-17 16:15:20.031512+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>29141</t>
+          <t>31201</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
+          <t>법제처, 추석 명절을 맞아 공주산성시장 방문</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=157132&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -911,39 +911,39 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-11 15:00:20.077861+09:00</t>
+          <t>2026-09-16 15:15:18.945495+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>27851</t>
+          <t>29141</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
+          <t>법제처, 추석맞이 아동양육시설 봉사활동, 따뜻한 나눔 실천</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -953,39 +953,39 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-08 13:30:19.671650+09:00</t>
+          <t>2026-09-11 15:00:20.077861+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>27461</t>
+          <t>27851</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>법제처, 제3회 특별성과 포상 수여</t>
+          <t>불합리한 행정법령 전수조사 첫 성과, 국토교통부 소관 법령 일괄정비안 국무회의 의결</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156753&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -995,39 +995,39 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-07 14:00:19.985373+09:00</t>
+          <t>2026-09-08 13:30:19.671650+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>25671</t>
+          <t>27461</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
+          <t>법제처, 제3회 특별성과 포상 수여</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156690&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1037,39 +1037,39 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-03 10:15:21.147736+09:00</t>
+          <t>2026-09-07 14:00:19.985373+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>24842</t>
+          <t>25671</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
+          <t>2027년도 법제처 예산안 700억 원 편성, 올해 대비 15.6% 증가</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156497&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1079,29 +1079,29 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-09-01 10:00:21.340393+09:00</t>
+          <t>2026-09-03 10:15:21.147736+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>24841</t>
+          <t>24842</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
+          <t>소방공무원 현장 대응 손해배상 보장 강화 및 개인정보 유출 대응 의무 대폭 확대</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156384&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1133,27 +1133,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>23411</t>
+          <t>24841</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
+          <t>Strengthening Damage Compensation Guarantee System for Firefighters' On-Site Response</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156385&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>법령정비지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1163,34 +1163,34 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2026-08-28 15:15:21.414160+09:00</t>
+          <t>2026-09-01 10:00:21.340393+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>23231</t>
+          <t>23411</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
+          <t>법제처, 미래 신기술과 인공지능(AI) 활용 관련 토론의 장 열어</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156162&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>법제자문1담당관</t>
+          <t>법령정비지원과</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1205,39 +1205,39 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-08-28 10:45:20.917220+09:00</t>
+          <t>2026-08-28 15:15:21.414160+09:00</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>14381</t>
+          <t>23231</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
+          <t>법제처, 공공기관 법제 지원 강화를 위한 수도권ㆍ강원권 현장설명회 개최</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=156157&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>법제자문1담당관</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1247,39 +1247,39 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2026-08-06 15:00:21.280220+09:00</t>
+          <t>2026-08-28 10:45:20.917220+09:00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>14121</t>
+          <t>14381</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>법제로 완성하는 국가대전환</t>
+          <t>제2회 법령데이터 활용 아이디어 공모전 시상식 개최</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154906&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>기획재정담당관실</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1289,39 +1289,39 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-08-06 08:30:20.431542+09:00</t>
+          <t>2026-08-06 15:00:21.280220+09:00</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12952</t>
+          <t>14121</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
+          <t>법제로 완성하는 국가대전환</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154855&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>기획재정담당관실</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1331,29 +1331,29 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>2026-08-03 10:00:19.612801+09:00</t>
+          <t>2026-08-06 08:30:20.431542+09:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12951</t>
+          <t>12952</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
+          <t>아동학대는 심층 분석, 저작권 침해는 강력 대응... 권익 보호와 산업 경쟁력 동시 강화</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154664&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1385,27 +1385,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11761</t>
+          <t>12951</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
+          <t>In-Depth Analysis of Child Abuse and Stronger Action against Copyright Infringement...</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154665&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>법제교육과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1415,34 +1415,34 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-07-31 11:00:19.812863+09:00</t>
+          <t>2026-08-03 10:00:19.612801+09:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11711</t>
+          <t>11761</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
+          <t>‘이론에서 실무로’ 제34기 법제처 실무수습 성황리에 마쳐</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154410&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법제교육과</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1457,39 +1457,39 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>2026-07-31 09:45:20.988339+09:00</t>
+          <t>2026-07-31 11:00:19.812863+09:00</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11311</t>
+          <t>11711</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>범정부 형벌 합리화 추진단 공식 출범</t>
+          <t>우리 지역 필수 자치법규 마련 현황, 국가법령정보센터에서 한눈에 확인!</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154405&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>파견</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1499,39 +1499,39 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>2026-07-30 10:00:20.929689+09:00</t>
+          <t>2026-07-31 09:45:20.988339+09:00</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>4471</t>
+          <t>11311</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
+          <t>범정부 형벌 합리화 추진단 공식 출범</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=154313&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>파견</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1541,39 +1541,39 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>2026-07-13 13:15:20.449920+09:00</t>
+          <t>2026-07-30 10:00:20.929689+09:00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1511</t>
+          <t>4471</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
+          <t>공무원이 직접 만든 ‘AI 법령 비서’ 시범 개시</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152980&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1583,39 +1583,39 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>2026-07-06 10:00:28.103718+09:00</t>
+          <t>2026-07-13 13:15:20.449920+09:00</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>1511</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
+          <t>법제처, 역대 처장ㆍ차장 초청 간담회 개최</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152615&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>법제교류협력담당관실</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1625,39 +1625,39 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2026-07-03 15:15:21.972107+09:00</t>
+          <t>2026-07-06 10:00:28.103718+09:00</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>491</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
+          <t>법제처, 한반도 환경위기 공동 대응을 위한 관학연 공동학술대회 개최</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152490&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>법제교류협력담당관실</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1667,29 +1667,29 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026-07-02 13:14:25.972950+09:00</t>
+          <t>2026-07-03 15:15:21.972107+09:00</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
+          <t>해수욕장 불꽃놀이는 허용, 일상 범죄와 소비자 피해는 철저히 방어!</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152381&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1721,27 +1721,27 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
+          <t>Permitting Beach Fireworks, While Strictly Preventing Crime Occurrence and Consumer Harm</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152382&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>운영지원과</t>
+          <t>대변인실</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1763,27 +1763,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
+          <t>법제처, ‘호국보훈의 달’ 맞아 광주보훈병원 국가유공자 위문</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152193&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>국가법령정보센터</t>
+          <t>운영지원과</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1805,27 +1805,27 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
+          <t>법제처, 생성형 AI 기반 대국민 법령검색 서비스 전환 추진</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152053&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>법령정비총괄과</t>
+          <t>국가법령정보센터</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1847,27 +1847,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
+          <t>청년 창업 활성화를 위한 법ㆍ제도 개선, 현장에서 답을 찾다</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=152008&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>자치법제지원과</t>
+          <t>법령정비총괄과</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1889,27 +1889,27 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
+          <t>법제처, 5극3특시대 지방정부의 자율성 확보를 위한 법제 개선의 장 열어</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151899&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>법령정보총괄과</t>
+          <t>자치법제지원과</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1931,27 +1931,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
+          <t>법제처, 국내 거주 외국인의 정착 지원 위한 맞춤형 생활법령 서비스 강화</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151696&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>혁신행정감사담당관실</t>
+          <t>법령정보총괄과</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1973,27 +1973,27 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+          <t>법제처, 기관 내 갑질 근절을 위한 ‘안심 상담ㆍ신고 노무사’ 제도 운영</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=151297&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>대변인실</t>
+          <t>혁신행정감사담당관실</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2015,40 +2015,82 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>New Laws will Take Effect to Protect Citizens and Promote Industries</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150887&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>대변인실</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2026-07-02 13:14:25.972950+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>자율주행 규제 합리화, 해외직구 안전 강화 등 국민보호 · 산업지원 새 법령 시행</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>https://www.moleg.go.kr/board.es?mid=a10501000000&amp;bid=0048&amp;act=view&amp;list_no=150819&amp;tag=&amp;pageCntBySelf=10&amp;nPage=1&amp;keyField=&amp;keyWord=&amp;cg_code=</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>대변인실</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>2026-07-02 13:14:25.972950+09:00</t>
         </is>

</xml_diff>